<commit_message>
getcensus v 3.0.0 (#78)
</commit_message>
<xml_diff>
--- a/docs/resources/doc_tables.xlsx
+++ b/docs/resources/doc_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\czippel\Documents\GitHub\getcensus\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClaireZippel\Documents\GitHub\getcensus\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBABDC8-1CD6-4B51-9119-1F7CE65E54AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AEE615-1E7C-4673-8109-8BABFDB122F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{614A9CB4-755C-45CD-BCD3-7F2BDDFCA0D2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{614A9CB4-755C-45CD-BCD3-7F2BDDFCA0D2}"/>
   </bookViews>
   <sheets>
     <sheet name="geographies" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="116">
   <si>
     <t>Name</t>
   </si>
@@ -176,9 +176,6 @@
     <t>statefips</t>
   </si>
   <si>
-    <t>†</t>
-  </si>
-  <si>
     <t>Code</t>
   </si>
   <si>
@@ -290,9 +287,6 @@
     <t>State Designated Tribal Statistical Area</t>
   </si>
   <si>
-    <t xml:space="preserve"> Hawaiian Home Land</t>
-  </si>
-  <si>
     <t>Not in metropolitan or micropolitan statistical area</t>
   </si>
   <si>
@@ -365,38 +359,194 @@
     <t>Population by income-to-poverty ratio</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>&lt;strong&gt;statefips&lt;/strong&gt;, countyfips</t>
-  </si>
-  <si>
-    <t>&lt;strong&gt;statefips&lt;/strong&gt;, &lt;strong&gt;countyfips&lt;/strong&gt;</t>
-  </si>
-  <si>
-    <t>&lt;strong&gt;statefips&lt;/strong&gt;</t>
-  </si>
-  <si>
-    <t>Housing characteristics, including housing costs*</t>
-  </si>
-  <si>
-    <t>Detailed renter housing cost burden*</t>
-  </si>
-  <si>
-    <t>statefips&lt;sup&gt;‡&lt;/sup&gt;</t>
+    <t>**statefips**, countyfips</t>
+  </si>
+  <si>
+    <t>**statefips**, **countyfips**</t>
+  </si>
+  <si>
+    <t>**statefips**</t>
+  </si>
+  <si>
+    <t>Hawaiian Home Land</t>
+  </si>
+  <si>
+    <r>
+      <t>Available with `</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>geography()`</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> *</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>us*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, *</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>region*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, *</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>division*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or *</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>state*</t>
+    </r>
+  </si>
+  <si>
+    <t>Availability</t>
+  </si>
+  <si>
+    <r>
+      <t>Available with `</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>geography(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>us</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>)`</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> only</t>
+    </r>
+  </si>
+  <si>
+    <t>Detailed renter housing cost burden</t>
+  </si>
+  <si>
+    <t>Housing characteristics, including housing costs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -440,9 +590,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -480,7 +630,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -586,7 +736,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -728,7 +878,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -736,260 +886,239 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F240D3E0-4FF9-4926-B14C-70DCEF4D2853}">
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
         <v>109</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
         <v>109</v>
       </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
         <v>109</v>
       </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" t="s">
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
       <c r="B22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
       <c r="B23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
       <c r="B24" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>26</v>
+      </c>
       <c r="B25" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1001,173 +1130,232 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAC423CC-ED26-4BD0-88E5-4652E112A278}">
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="43.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.90625" style="1"/>
+    <col min="3" max="3" width="43.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="C12" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" s="1">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>113</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="1" t="s">
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="1" t="s">
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="C17" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" s="1" t="s">
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="1" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>43</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>77</v>
+      <c r="C20" s="1" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1178,114 +1366,114 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54DD25C4-A271-4D4C-8519-DA5D6FC2E821}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="73.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="73.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
         <v>87</v>
       </c>
-      <c r="B3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B5" t="s">
         <v>88</v>
       </c>
-      <c r="B4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
         <v>89</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
         <v>91</v>
       </c>
-      <c r="B6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
         <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>94</v>
       </c>
       <c r="B9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
         <v>95</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B12" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
         <v>97</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>